<commit_message>
Added ability to generate separate deviations figures
</commit_message>
<xml_diff>
--- a/test/Figure Data.xlsx
+++ b/test/Figure Data.xlsx
@@ -8,22 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deaco\PycharmProjects\FigureGenerator\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A033BD-A344-414D-A36F-BDF48DCAED21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC807817-4839-4CBA-8FE8-6EA1C362E487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="13583" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DyOHCO_3" sheetId="1" r:id="rId1"/>
-    <sheet name="SmOHCO_3" sheetId="2" r:id="rId2"/>
+    <sheet name="DyOHCO_3⋅0.008H_2O" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="A_Cp_Cv">#REF!</definedName>
-    <definedName name="ad_sub">#REF!</definedName>
-    <definedName name="Al_sub">#REF!</definedName>
-    <definedName name="Cu_sub">#REF!</definedName>
-    <definedName name="Ngr_sub">#REF!</definedName>
-    <definedName name="Other_sub">#REF!</definedName>
-    <definedName name="scalingfactor">#REF!</definedName>
+    <definedName name="A_Cp_Cv">DyOHCO_3⋅0.008H_2O!$T$31</definedName>
+    <definedName name="ad_sub">DyOHCO_3⋅0.008H_2O!$O$2</definedName>
+    <definedName name="Al_sub">DyOHCO_3⋅0.008H_2O!$O$6</definedName>
+    <definedName name="Cu_sub">DyOHCO_3⋅0.008H_2O!$O$4</definedName>
+    <definedName name="Ngr_sub">DyOHCO_3⋅0.008H_2O!$O$8</definedName>
+    <definedName name="Other_sub">DyOHCO_3⋅0.008H_2O!$O$10</definedName>
+    <definedName name="scalingfactor">DyOHCO_3⋅0.008H_2O!$L$6</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -96,9 +96,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3024,2756 +3023,2644 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0456B3C2-D951-4FC7-9524-B97BA87CB819}">
-  <dimension ref="A1:E238"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F91FB640-02F6-4746-BB49-68F43BA33118}">
+  <dimension ref="A1:F224"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="19.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.06640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.46484375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.53125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.53125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.3984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.06640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2">
+        <v>1.7</v>
+      </c>
+      <c r="B2">
+        <v>4.575958647677191</v>
+      </c>
+      <c r="D2">
+        <v>1.82854543333333</v>
+      </c>
+      <c r="E2">
+        <v>3.9028740403415543</v>
+      </c>
+      <c r="F2">
+        <v>1.0104516777686308</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A3">
+        <v>1.8</v>
+      </c>
+      <c r="B3">
+        <v>4.0039436855439519</v>
+      </c>
+      <c r="D3">
+        <v>1.90187603333333</v>
+      </c>
+      <c r="E3">
+        <v>3.5193470332411447</v>
+      </c>
+      <c r="F3">
+        <v>-0.63458308712012546</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4">
+        <v>1.9</v>
+      </c>
+      <c r="B4">
+        <v>3.5494475485554084</v>
+      </c>
+      <c r="D4">
+        <v>1.97795963333333</v>
+      </c>
+      <c r="E4">
+        <v>3.208857800469211</v>
+      </c>
+      <c r="F4">
+        <v>-1.4472571990911749</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5">
+        <v>3.1809195204389202</v>
+      </c>
+      <c r="D5">
+        <v>2.0595674000000002</v>
+      </c>
+      <c r="E5">
+        <v>2.9441467081165777</v>
+      </c>
+      <c r="F5">
+        <v>-1.6342309524622685</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A6">
+        <v>2.1</v>
+      </c>
+      <c r="B6">
+        <v>2.8767273910504136</v>
+      </c>
+      <c r="D6">
+        <v>2.1470653333333298</v>
+      </c>
+      <c r="E6">
+        <v>2.7581543678396288</v>
+      </c>
+      <c r="F6">
+        <v>0.24850522997303809</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A7">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B7">
+        <v>2.6216937153683055</v>
+      </c>
+      <c r="D7">
+        <v>2.2384766666666698</v>
+      </c>
+      <c r="E7">
+        <v>2.6003855563446412</v>
+      </c>
+      <c r="F7">
+        <v>2.6096141258920245</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A8">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="B8">
+        <v>2.4049410699768066</v>
+      </c>
+      <c r="D8">
+        <v>2.3344990666666701</v>
+      </c>
+      <c r="E8">
+        <v>2.3995731903574025</v>
+      </c>
+      <c r="F8">
+        <v>2.6539669748698831</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A9">
+        <v>2.4</v>
+      </c>
+      <c r="B9">
+        <v>2.2185190115089903</v>
+      </c>
+      <c r="D9">
+        <v>2.4335296666666699</v>
+      </c>
+      <c r="E9">
+        <v>2.1892651907478573</v>
+      </c>
+      <c r="F9">
+        <v>1.2740056496125156</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A10">
+        <v>2.5</v>
+      </c>
+      <c r="B10">
+        <v>2.0565096229109572</v>
+      </c>
+      <c r="D10">
+        <v>2.5372245000000002</v>
+      </c>
+      <c r="E10">
+        <v>1.9667217086579443</v>
+      </c>
+      <c r="F10">
+        <v>-1.737446658746306</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A11">
+        <v>2.6</v>
+      </c>
+      <c r="B11">
+        <v>1.9144328324523199</v>
+      </c>
+      <c r="D11">
+        <v>2.6510762333333302</v>
+      </c>
+      <c r="E11">
+        <v>1.8314122786904592</v>
+      </c>
+      <c r="F11">
+        <v>-0.91962891551409465</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A12">
+        <v>2.7</v>
+      </c>
+      <c r="B12">
+        <v>1.7888434890757463</v>
+      </c>
+      <c r="D12">
+        <v>2.7674069000000001</v>
+      </c>
+      <c r="E12">
+        <v>1.7001635552067345</v>
+      </c>
+      <c r="F12">
+        <v>-0.69796483158300315</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A13">
+        <v>2.8</v>
+      </c>
+      <c r="B13">
+        <v>1.6770535080770224</v>
+      </c>
+      <c r="D13">
+        <v>2.8878344333333299</v>
+      </c>
+      <c r="E13">
+        <v>1.5812182712226415</v>
+      </c>
+      <c r="F13">
+        <v>-0.46175113797319511</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A14">
+        <v>2.9</v>
+      </c>
+      <c r="B14">
+        <v>1.5769370804330569</v>
+      </c>
+      <c r="D14">
+        <v>3.0171441666666698</v>
+      </c>
+      <c r="E14">
+        <v>1.4674119903118235</v>
+      </c>
+      <c r="F14">
+        <v>-0.32755242784409988</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A15">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="B15">
+        <v>1.4867919864104289</v>
+      </c>
+      <c r="D15">
+        <v>3.1563782666666702</v>
+      </c>
+      <c r="E15">
+        <v>1.3537941585303315</v>
+      </c>
+      <c r="F15">
+        <v>-0.64737518043857378</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A16">
+        <v>3.1</v>
+      </c>
+      <c r="B16">
+        <v>1.4052394077669867</v>
+      </c>
+      <c r="D16">
+        <v>3.3007199333333301</v>
+      </c>
+      <c r="E16">
+        <v>1.2492790471389885</v>
+      </c>
+      <c r="F16">
+        <v>-1.0963662522559028</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A17">
+        <v>3.2</v>
+      </c>
+      <c r="B17">
+        <v>1.3311505528063687</v>
+      </c>
+      <c r="D17">
+        <v>3.4509051999999998</v>
+      </c>
+      <c r="E17">
+        <v>1.1566741553788751</v>
+      </c>
+      <c r="F17">
+        <v>-1.334441433664914</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A18">
+        <v>3.3</v>
+      </c>
+      <c r="B18">
+        <v>1.2635922187269941</v>
+      </c>
+      <c r="D18">
+        <v>3.6052875666666702</v>
+      </c>
+      <c r="E18">
+        <v>1.0776528297993815</v>
+      </c>
+      <c r="F18">
+        <v>-1.1571081774943495</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A19">
+        <v>3.4</v>
+      </c>
+      <c r="B19">
+        <v>1.2017859068772838</v>
+      </c>
+      <c r="D19">
+        <v>3.7657816999999998</v>
+      </c>
+      <c r="E19">
+        <v>1.0108247728493729</v>
+      </c>
+      <c r="F19">
+        <v>-0.42998846976220306</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A20">
+        <v>3.5</v>
+      </c>
+      <c r="B20">
+        <v>1.145076759545379</v>
+      </c>
+      <c r="D20">
+        <v>3.9335581333333298</v>
+      </c>
+      <c r="E20">
+        <v>0.95067710637706804</v>
+      </c>
+      <c r="F20">
+        <v>0.48056161136418102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A21">
+        <v>3.6</v>
+      </c>
+      <c r="B21">
+        <v>1.0929096991427187</v>
+      </c>
+      <c r="D21">
+        <v>4.1113730000000004</v>
+      </c>
+      <c r="E21">
+        <v>0.89694870038084196</v>
+      </c>
+      <c r="F21">
+        <v>1.7097760206242834</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A22">
+        <v>3.7</v>
+      </c>
+      <c r="B22">
+        <v>1.044810908906586</v>
+      </c>
+      <c r="D22">
+        <v>4.2929111666666699</v>
+      </c>
+      <c r="E22">
+        <v>0.83497393671513387</v>
+      </c>
+      <c r="F22">
+        <v>1.2881677384297088</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A23">
+        <v>3.8</v>
+      </c>
+      <c r="B23">
+        <v>1.0003733176688518</v>
+      </c>
+      <c r="D23">
+        <v>4.4838927000000002</v>
+      </c>
+      <c r="E23">
+        <v>0.77627594438802427</v>
+      </c>
+      <c r="F23">
+        <v>0.63150112429238203</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A24">
+        <v>3.9</v>
+      </c>
+      <c r="B24">
+        <v>0.95924511684151348</v>
+      </c>
+      <c r="D24">
+        <v>4.6822281333333304</v>
+      </c>
+      <c r="E24">
+        <v>0.72502028352792425</v>
+      </c>
+      <c r="F24">
+        <v>0.21310680340909433</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A25">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A2">
-        <v>1.8315676333333299</v>
-      </c>
-      <c r="B2">
-        <v>0.14366149946749246</v>
-      </c>
-      <c r="C2">
-        <v>0.10066360180235061</v>
-      </c>
-      <c r="D2" s="1">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A3">
-        <v>1.9069596666666699</v>
-      </c>
-      <c r="B3">
-        <v>0.13355090190962454</v>
-      </c>
-      <c r="C3">
-        <v>-0.48474698066034222</v>
-      </c>
-      <c r="D3">
-        <v>0.4</v>
-      </c>
-      <c r="E3">
-        <v>0.48612798140597463</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A4">
-        <v>1.9829910666666699</v>
-      </c>
-      <c r="B4">
-        <v>0.12470464989655575</v>
-      </c>
-      <c r="C4">
-        <v>-0.84322520243880184</v>
-      </c>
-      <c r="D4">
-        <v>0.5</v>
-      </c>
-      <c r="E4">
-        <v>0.55464742087872487</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A5">
-        <v>2.0647967</v>
-      </c>
-      <c r="B5">
-        <v>0.11648565751098637</v>
-      </c>
-      <c r="C5">
-        <v>-0.97965094344872605</v>
-      </c>
-      <c r="D5">
-        <v>0.6</v>
-      </c>
-      <c r="E5">
-        <v>0.55025181993974936</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A6">
-        <v>2.1517277333333298</v>
-      </c>
-      <c r="B6">
-        <v>0.11110716173248608</v>
-      </c>
-      <c r="C6">
-        <v>1.0494187296685118</v>
-      </c>
-      <c r="D6">
-        <v>0.7</v>
-      </c>
-      <c r="E6">
-        <v>0.51101932392671323</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A7">
-        <v>2.2424008999999998</v>
-      </c>
-      <c r="B7">
-        <v>0.10486568102156452</v>
-      </c>
-      <c r="C7">
-        <v>1.9546547530649345</v>
-      </c>
-      <c r="D7">
-        <v>0.8</v>
-      </c>
-      <c r="E7">
-        <v>0.45984921858287287</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A8">
-        <v>2.3384744666666699</v>
-      </c>
-      <c r="B8">
-        <v>9.930068152812456E-2</v>
-      </c>
-      <c r="C8">
-        <v>3.1908261871761243</v>
-      </c>
-      <c r="D8">
-        <v>0.9</v>
-      </c>
-      <c r="E8">
-        <v>0.40795066165005461</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A9">
-        <v>2.4365066999999998</v>
-      </c>
-      <c r="B9">
-        <v>9.2431221350331313E-2</v>
-      </c>
-      <c r="C9">
-        <v>2.3574879085623071</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>0.36004192154729731</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A10">
-        <v>2.540489</v>
-      </c>
-      <c r="B10">
-        <v>8.2059821964582211E-2</v>
-      </c>
-      <c r="C10">
-        <v>-3.2535971991426771</v>
-      </c>
-      <c r="D10">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="E10">
-        <v>0.31766578333740203</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A11">
-        <v>2.6542099000000001</v>
-      </c>
-      <c r="B11">
-        <v>7.8209769438626564E-2</v>
-      </c>
-      <c r="C11">
-        <v>-1.8117580529262076</v>
-      </c>
-      <c r="D11">
-        <v>1.2</v>
-      </c>
-      <c r="E11">
-        <v>0.28093711073898314</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A12">
-        <v>2.7702634666666701</v>
-      </c>
-      <c r="B12">
-        <v>7.4650641900338252E-2</v>
-      </c>
-      <c r="C12">
-        <v>-0.68020553373645398</v>
-      </c>
-      <c r="D12">
-        <v>1.3</v>
-      </c>
-      <c r="E12">
-        <v>0.24939404838323104</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A13">
-        <v>2.89066926666667</v>
-      </c>
-      <c r="B13">
-        <v>7.1245181175657118E-2</v>
-      </c>
-      <c r="C13">
-        <v>1.6446872189553721E-2</v>
-      </c>
-      <c r="D13">
-        <v>1.4</v>
-      </c>
-      <c r="E13">
-        <v>0.22239250732519278</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A14">
-        <v>3.0177019999999999</v>
-      </c>
-      <c r="B14">
-        <v>6.7536181527403469E-2</v>
-      </c>
-      <c r="C14">
-        <v>-0.38699368528154565</v>
-      </c>
-      <c r="D14">
-        <v>1.5</v>
-      </c>
-      <c r="E14">
-        <v>0.19927910479017466</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A15">
-        <v>3.1550304666666702</v>
-      </c>
-      <c r="B15">
-        <v>6.4064307922946387E-2</v>
-      </c>
-      <c r="C15">
-        <v>-1.1475304959513244</v>
-      </c>
-      <c r="D15">
-        <v>1.6</v>
-      </c>
-      <c r="E15">
-        <v>0.17945973839622037</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A16">
-        <v>3.3000995333333298</v>
-      </c>
-      <c r="B16">
-        <v>6.1088788005754596E-2</v>
-      </c>
-      <c r="C16">
-        <v>-2.0544979010167594</v>
-      </c>
-      <c r="D16">
-        <v>1.7</v>
-      </c>
-      <c r="E16">
-        <v>0.16242046464662571</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A17">
-        <v>3.4500281333333298</v>
-      </c>
-      <c r="B17">
-        <v>5.9645550540135324E-2</v>
-      </c>
-      <c r="C17">
-        <v>-1.4825994658150572</v>
-      </c>
-      <c r="D17">
-        <v>1.8</v>
-      </c>
-      <c r="E17">
-        <v>0.14772764427526378</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A18">
-        <v>3.6047310666666701</v>
-      </c>
-      <c r="B18">
-        <v>5.874357875753132E-2</v>
-      </c>
-      <c r="C18">
-        <v>-0.97115061532490865</v>
-      </c>
-      <c r="D18">
-        <v>1.9</v>
-      </c>
-      <c r="E18">
-        <v>0.13501997909173036</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A19">
-        <v>3.7650030999999999</v>
-      </c>
-      <c r="B19">
-        <v>5.8407851664150627E-2</v>
-      </c>
-      <c r="C19">
-        <v>-0.48792078723992199</v>
-      </c>
-      <c r="D19">
-        <v>2</v>
-      </c>
-      <c r="E19">
-        <v>0.12399819809719353</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A20">
-        <v>3.9338652000000001</v>
-      </c>
-      <c r="B20">
-        <v>5.8432270375760341E-2</v>
-      </c>
-      <c r="C20">
-        <v>-0.42617979456738697</v>
-      </c>
-      <c r="D20">
-        <v>2.1</v>
-      </c>
-      <c r="E20">
-        <v>0.11441488531477748</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A21">
-        <v>4.1080465666666699</v>
-      </c>
-      <c r="B21">
-        <v>5.9696029153487824E-2</v>
-      </c>
-      <c r="C21">
-        <v>0.64415856781810366</v>
-      </c>
-      <c r="D21">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="E21">
-        <v>0.10606540943103851</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A22">
-        <v>4.2899865000000004</v>
-      </c>
-      <c r="B22">
-        <v>6.0304442527119216E-2</v>
-      </c>
-      <c r="C22">
-        <v>-0.53239795855417293</v>
-      </c>
-      <c r="D22">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="E22">
-        <v>9.878021572920534E-2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A23">
-        <v>4.48162136666667</v>
-      </c>
-      <c r="B23">
-        <v>6.3295415259645604E-2</v>
-      </c>
-      <c r="C23">
-        <v>0.95855064425283965</v>
-      </c>
-      <c r="D23">
-        <v>2.4</v>
-      </c>
-      <c r="E23">
-        <v>9.2418439211778072E-2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A24">
-        <v>4.6795206333333299</v>
-      </c>
-      <c r="B24">
-        <v>6.4197233326772546E-2</v>
-      </c>
-      <c r="C24">
-        <v>-2.0416390279612924</v>
-      </c>
-      <c r="D24">
-        <v>2.5</v>
-      </c>
-      <c r="E24">
-        <v>8.6862683823014791E-2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A25">
-        <v>4.89147626666667</v>
-      </c>
       <c r="B25">
-        <v>6.9292874946174907E-2</v>
-      </c>
-      <c r="C25">
-        <v>-8.1044813379646613E-2</v>
+        <v>0.92112059602108753</v>
       </c>
       <c r="D25">
-        <v>2.6</v>
+        <v>4.8907178333333299</v>
       </c>
       <c r="E25">
-        <v>8.2014784439336352E-2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.68421954410420249</v>
+      </c>
+      <c r="F25">
+        <v>0.64918791577728741</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26">
-        <v>5.10602703333333</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="B26">
-        <v>7.4295946918761457E-2</v>
-      </c>
-      <c r="C26">
-        <v>0.39123712353443024</v>
+        <v>0.88573276799547718</v>
       </c>
       <c r="D26">
-        <v>2.7</v>
+        <v>5.1063758000000004</v>
       </c>
       <c r="E26">
-        <v>7.7792376799752358E-2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.64467652890067562</v>
+      </c>
+      <c r="F26">
+        <v>0.58644588053016322</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A27">
-        <v>5.3356702</v>
+        <v>4.2</v>
       </c>
       <c r="B27">
-        <v>8.1361817168356804E-2</v>
-      </c>
-      <c r="C27">
-        <v>1.8657481190084908</v>
+        <v>0.8528473869274058</v>
       </c>
       <c r="D27">
-        <v>2.8</v>
+        <v>5.3376549000000004</v>
       </c>
       <c r="E27">
-        <v>7.4126122609671483E-2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.61208217083741456</v>
+      </c>
+      <c r="F27">
+        <v>1.1021871514928938</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28">
-        <v>5.5707685666666702</v>
+        <v>4.3</v>
       </c>
       <c r="B28">
-        <v>9.1907718124384086E-2</v>
-      </c>
-      <c r="C28">
-        <v>5.8603293717505185</v>
+        <v>0.82225806035049664</v>
       </c>
       <c r="D28">
-        <v>2.9</v>
+        <v>5.5734078333333299</v>
       </c>
       <c r="E28">
-        <v>7.0957462070779173E-2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.59301255903262717</v>
+      </c>
+      <c r="F28">
+        <v>3.131128578482214</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A29">
-        <v>5.8185852999999996</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="B29">
-        <v>0.10058348088579722</v>
-      </c>
-      <c r="C29">
-        <v>5.6688840417216202</v>
+        <v>0.79378222682264887</v>
       </c>
       <c r="D29">
-        <v>3</v>
+        <v>5.8199140666666702</v>
       </c>
       <c r="E29">
-        <v>6.8236789561675282E-2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.56545790340974611</v>
+      </c>
+      <c r="F29">
+        <v>3.0452500055681151</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30">
-        <v>6.0770588333333304</v>
+        <v>4.5</v>
       </c>
       <c r="B30">
-        <v>0.10797737500745912</v>
-      </c>
-      <c r="C30">
-        <v>2.761256872236785</v>
+        <v>0.76725782389974262</v>
       </c>
       <c r="D30">
-        <v>3.1</v>
+        <v>6.0764296</v>
       </c>
       <c r="E30">
-        <v>6.5921968506511983E-2</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.53069671412478236</v>
+      </c>
+      <c r="F30">
+        <v>0.74669703568760193</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31">
-        <v>6.3477586666666701</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="B31">
-        <v>0.11541530117714709</v>
-      </c>
-      <c r="C31">
-        <v>-1.1299435826325273</v>
+        <v>0.74254051060666237</v>
       </c>
       <c r="D31">
-        <v>3.2</v>
+        <v>6.3461751</v>
       </c>
       <c r="E31">
-        <v>6.3977118330150864E-2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.49800755967785021</v>
+      </c>
+      <c r="F31">
+        <v>-2.145050435279741</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A32">
-        <v>6.6268663333333304</v>
+        <v>4.7</v>
       </c>
       <c r="B32">
-        <v>0.12644771090288248</v>
-      </c>
-      <c r="C32">
-        <v>-2.8759903407272707</v>
+        <v>0.71950133838684049</v>
       </c>
       <c r="D32">
-        <v>3.3</v>
+        <v>6.6269736000000004</v>
       </c>
       <c r="E32">
-        <v>6.2371620071734267E-2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.48105140248325567</v>
+      </c>
+      <c r="F32">
+        <v>-2.9280970533582198</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A33">
-        <v>6.9221909666666699</v>
+        <v>4.8</v>
       </c>
       <c r="B33">
-        <v>0.14136216179197508</v>
-      </c>
-      <c r="C33">
-        <v>-3.2274997882116989</v>
+        <v>0.69802478716956806</v>
       </c>
       <c r="D33">
-        <v>3.4</v>
+        <v>6.9224245666666704</v>
       </c>
       <c r="E33">
-        <v>6.1079298168565818E-2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.4786594154067294</v>
+      </c>
+      <c r="F33">
+        <v>-1.6618277271473922</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A34">
-        <v>7.2263144333333296</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="B34">
-        <v>0.16193062287204305</v>
-      </c>
-      <c r="C34">
-        <v>-1.4256531306831475</v>
+        <v>0.67800710055033542</v>
       </c>
       <c r="D34">
-        <v>3.5</v>
+        <v>7.2297540666666702</v>
       </c>
       <c r="E34">
-        <v>6.0077744608935196E-2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.47723427356857517</v>
+      </c>
+      <c r="F34">
+        <v>-1.1645688438850965</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A35">
-        <v>7.5521943666666704</v>
+        <v>5</v>
       </c>
       <c r="B35">
-        <v>0.18574013892699895</v>
-      </c>
-      <c r="C35">
-        <v>-0.10171469811490814</v>
+        <v>0.65935486747102579</v>
       </c>
       <c r="D35">
-        <v>3.6</v>
+        <v>7.54865503333333</v>
       </c>
       <c r="E35">
-        <v>5.9347758523049354E-2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.48437642522710861</v>
+      </c>
+      <c r="F35">
+        <v>4.9000353346737142E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A36">
-        <v>7.8858912333333304</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="B36">
-        <v>0.21170286502986757</v>
-      </c>
-      <c r="C36">
-        <v>0.55881831014801475</v>
+        <v>0.64198380819179446</v>
       </c>
       <c r="D36">
-        <v>3.7</v>
+        <v>7.8872839333333298</v>
       </c>
       <c r="E36">
-        <v>5.8872879706991406E-2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.48980714276206483</v>
+      </c>
+      <c r="F36">
+        <v>-0.26507278938071172</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A37">
-        <v>8.2345660333333299</v>
+        <v>5.2</v>
       </c>
       <c r="B37">
-        <v>0.2379588705186009</v>
-      </c>
-      <c r="C37">
-        <v>-0.42325509091386959</v>
+        <v>0.62581773048541978</v>
       </c>
       <c r="D37">
-        <v>3.8</v>
+        <v>8.2268690000000007</v>
       </c>
       <c r="E37">
-        <v>5.8638998859828428E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.50380242443097223</v>
+      </c>
+      <c r="F37">
+        <v>3.0090778623693446E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A38">
-        <v>8.59809816666667</v>
+        <v>5.3</v>
       </c>
       <c r="B38">
-        <v>0.27066870254938841</v>
-      </c>
-      <c r="C38">
-        <v>-0.40059919816642292</v>
+        <v>0.61078762839246836</v>
       </c>
       <c r="D38">
-        <v>3.9</v>
+        <v>8.6019975666666699</v>
       </c>
       <c r="E38">
-        <v>5.8634030702449033E-2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.52364527624067037</v>
+      </c>
+      <c r="F38">
+        <v>-2.1542533041796093E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A39">
-        <v>8.9786187666666706</v>
+        <v>5.4</v>
       </c>
       <c r="B39">
-        <v>0.30825146275868293</v>
-      </c>
-      <c r="C39">
-        <v>-0.4584881031403128</v>
+        <v>0.59683090095152025</v>
       </c>
       <c r="D39">
-        <v>4</v>
+        <v>8.9781489000000008</v>
       </c>
       <c r="E39">
-        <v>5.8847638831364478E-2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.55097274736729862</v>
+      </c>
+      <c r="F39">
+        <v>0.11083172740685948</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40">
-        <v>9.3816985666666692</v>
+        <v>5.5</v>
       </c>
       <c r="B40">
-        <v>0.35441076215412542</v>
-      </c>
-      <c r="C40">
-        <v>0.10341718719159441</v>
+        <v>0.58389067236370806</v>
       </c>
       <c r="D40">
-        <v>4.0999999999999996</v>
+        <v>9.3774207000000001</v>
       </c>
       <c r="E40">
-        <v>5.9271003293062556E-2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.58285112327809629</v>
+      </c>
+      <c r="F40">
+        <v>-0.46349251748614972</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41">
-        <v>9.7936441666666703</v>
+        <v>5.6</v>
       </c>
       <c r="B41">
-        <v>0.40780036092648575</v>
-      </c>
-      <c r="C41">
-        <v>0.91743999467616755</v>
+        <v>0.57191519829285098</v>
       </c>
       <c r="D41">
-        <v>4.2</v>
+        <v>9.7931760666666694</v>
       </c>
       <c r="E41">
-        <v>5.9896623563043309E-2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.63075224322024348</v>
+      </c>
+      <c r="F41">
+        <v>0.15167042762629657</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A42">
-        <v>10.240683333333299</v>
+        <v>5.7</v>
       </c>
       <c r="B42">
-        <v>0.45934452659729341</v>
-      </c>
-      <c r="C42">
-        <v>-1.0123313438681001</v>
+        <v>0.56085734561529021</v>
       </c>
       <c r="D42">
-        <v>4.3</v>
+        <v>10.240432</v>
       </c>
       <c r="E42">
-        <v>6.0718150970868807E-2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.683509252584655</v>
+      </c>
+      <c r="F42">
+        <v>-0.36485302911915962</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A43">
-        <v>10.694829333333301</v>
+        <v>5.8</v>
       </c>
       <c r="B43">
-        <v>0.53426266109136966</v>
-      </c>
-      <c r="C43">
-        <v>0.34689912785940236</v>
+        <v>0.55067413505042007</v>
       </c>
       <c r="D43">
-        <v>4.4000000000000004</v>
+        <v>10.695046</v>
       </c>
       <c r="E43">
-        <v>6.1730245700582553E-2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.75587295611193883</v>
+      </c>
+      <c r="F43">
+        <v>0.46681511394862651</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A44">
-        <v>11.171193333333299</v>
+        <v>5.9</v>
       </c>
       <c r="B44">
-        <v>0.60906228554209774</v>
-      </c>
-      <c r="C44">
-        <v>-0.37379689192735538</v>
+        <v>0.54132633782678086</v>
       </c>
       <c r="D44">
-        <v>4.5</v>
+        <v>11.169767999999999</v>
       </c>
       <c r="E44">
-        <v>6.2928454371032796E-2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.83336802290871359</v>
+      </c>
+      <c r="F44">
+        <v>0.21103327252476484</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A45">
-        <v>11.6670483333333</v>
+        <v>6</v>
       </c>
       <c r="B45">
-        <v>0.69990118236740351</v>
-      </c>
-      <c r="C45">
-        <v>-0.20494274742365381</v>
+        <v>0.53277811894928928</v>
       </c>
       <c r="D45">
-        <v>4.5999999999999996</v>
+        <v>11.666510000000001</v>
       </c>
       <c r="E45">
-        <v>6.4309104907028194E-2</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.92695249143948877</v>
+      </c>
+      <c r="F45">
+        <v>0.15683068768960878</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A46">
-        <v>12.185591000000001</v>
+        <v>6.1</v>
       </c>
       <c r="B46">
-        <v>0.80240299192201348</v>
-      </c>
-      <c r="C46">
-        <v>-0.21123338474164371</v>
+        <v>0.52499672079304005</v>
       </c>
       <c r="D46">
-        <v>4.7</v>
+        <v>12.184478</v>
       </c>
       <c r="E46">
-        <v>6.5869215984381294E-2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
+        <v>1.0377566760846391</v>
+      </c>
+      <c r="F46">
+        <v>0.23245528626728523</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A47">
-        <v>12.7254163333333</v>
+        <v>6.2</v>
       </c>
       <c r="B47">
-        <v>0.91485118085958461</v>
-      </c>
-      <c r="C47">
-        <v>-0.62146779974376909</v>
+        <v>0.51795218170708257</v>
       </c>
       <c r="D47">
-        <v>4.8</v>
+        <v>12.7233513333333</v>
       </c>
       <c r="E47">
-        <v>6.7606418796874748E-2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
+        <v>1.1604105946402707</v>
+      </c>
+      <c r="F47">
+        <v>-0.17905955707726812</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A48">
-        <v>13.288349666666701</v>
+        <v>6.3</v>
       </c>
       <c r="B48">
-        <v>1.0436808881656774</v>
-      </c>
-      <c r="C48">
-        <v>-0.828974985139034</v>
+        <v>0.51161708510622295</v>
       </c>
       <c r="D48">
-        <v>4.9000000000000004</v>
+        <v>13.2864033333333</v>
       </c>
       <c r="E48">
-        <v>6.951888927237547E-2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
+        <v>1.3068474232898517</v>
+      </c>
+      <c r="F48">
+        <v>-0.17032119459227546</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A49">
-        <v>13.87818</v>
+        <v>6.4</v>
       </c>
       <c r="B49">
-        <v>1.1979593945063289</v>
-      </c>
-      <c r="C49">
-        <v>-0.33113398709280328</v>
+        <v>0.50596633519083201</v>
       </c>
       <c r="D49">
-        <v>5</v>
+        <v>13.877641333333299</v>
       </c>
       <c r="E49">
-        <v>7.1605289175594083E-2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
+        <v>1.4780253963617609</v>
+      </c>
+      <c r="F49">
+        <v>3.3833312553195619E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A50">
-        <v>14.494600333333301</v>
+        <v>6.5</v>
       </c>
       <c r="B50">
-        <v>1.3716565962193783</v>
-      </c>
-      <c r="C50">
-        <v>7.0509931092340272E-2</v>
+        <v>0.50097695598825154</v>
       </c>
       <c r="D50">
-        <v>5.0999999999999996</v>
+        <v>14.494206999999999</v>
       </c>
       <c r="E50">
-        <v>7.3864714789714028E-2</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
+        <v>1.6682982317894677</v>
+      </c>
+      <c r="F50">
+        <v>0.13750843225722731</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A51">
-        <v>15.1363153333333</v>
+        <v>6.6</v>
       </c>
       <c r="B51">
-        <v>1.5567382044883171</v>
-      </c>
-      <c r="C51">
-        <v>-0.20151094470307421</v>
+        <v>0.49662791087417862</v>
       </c>
       <c r="D51">
-        <v>5.2</v>
+        <v>15.134926999999999</v>
       </c>
       <c r="E51">
-        <v>7.6296652078919822E-2</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
+        <v>1.8789364072530739</v>
+      </c>
+      <c r="F51">
+        <v>0.17160307652703349</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A52">
-        <v>15.642011666666701</v>
+        <v>6.7</v>
       </c>
       <c r="B52">
-        <v>1.7083044530432778</v>
-      </c>
-      <c r="C52">
-        <v>-0.60168199545954348</v>
+        <v>0.49289994012408894</v>
       </c>
       <c r="D52">
-        <v>5.3</v>
+        <v>15.639977999999999</v>
       </c>
       <c r="E52">
-        <v>7.8900937407217028E-2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
+        <v>2.0500070780340018</v>
+      </c>
+      <c r="F52">
+        <v>-0.10106817553889244</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A53">
-        <v>17.0947623333333</v>
+        <v>6.8</v>
       </c>
       <c r="B53">
-        <v>2.2180039878774624</v>
-      </c>
-      <c r="C53">
-        <v>-0.16749901395689082</v>
+        <v>0.48977541437600358</v>
       </c>
       <c r="D53">
-        <v>5.4</v>
+        <v>17.092874333333299</v>
       </c>
       <c r="E53">
-        <v>8.16777230326311E-2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
+        <v>2.6265495596910138</v>
+      </c>
+      <c r="F53">
+        <v>0.52937746600261026</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A54">
-        <v>18.6832836666667</v>
+        <v>6.9</v>
       </c>
       <c r="B54">
-        <v>2.8759795277579521</v>
-      </c>
-      <c r="C54">
-        <v>0.9032192426924992</v>
+        <v>0.48723820216699726</v>
       </c>
       <c r="D54">
-        <v>5.5</v>
+        <v>18.680372333333299</v>
       </c>
       <c r="E54">
-        <v>8.4627446715344654E-2</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
+        <v>3.351960351365038</v>
+      </c>
+      <c r="F54">
+        <v>1.1853825728346012</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A55">
-        <v>20.413724333333299</v>
+        <v>7</v>
       </c>
       <c r="B55">
-        <v>3.6610958511328597</v>
-      </c>
-      <c r="C55">
-        <v>0.98444510623577297</v>
+        <v>0.48527354994517613</v>
       </c>
       <c r="D55">
-        <v>5.6</v>
+        <v>20.4122016666667</v>
       </c>
       <c r="E55">
-        <v>8.7750804877961205E-2</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
+        <v>4.217874895438829</v>
+      </c>
+      <c r="F55">
+        <v>1.0465113865455415</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A56">
-        <v>22.3162423333333</v>
+        <v>7.1</v>
       </c>
       <c r="B56">
-        <v>4.6243666680152709</v>
-      </c>
-      <c r="C56">
-        <v>0.91781128484217722</v>
+        <v>0.48386797316325808</v>
       </c>
       <c r="D56">
-        <v>5.7</v>
+        <v>22.312722333333301</v>
       </c>
       <c r="E56">
-        <v>9.104872883940518E-2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
+        <v>5.2587379769181286</v>
+      </c>
+      <c r="F56">
+        <v>0.61434308469629961</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A57">
-        <v>24.3889213333333</v>
+        <v>7.2</v>
       </c>
       <c r="B57">
-        <v>5.7674919180914657</v>
-      </c>
-      <c r="C57">
-        <v>0.42734211062135641</v>
+        <v>0.4830091572350122</v>
       </c>
       <c r="D57">
-        <v>5.8</v>
+        <v>24.386292999999998</v>
       </c>
       <c r="E57">
-        <v>9.4522363713853835E-2</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
+        <v>6.489297151080029</v>
+      </c>
+      <c r="F57">
+        <v>4.9167371562984043E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A58">
-        <v>26.656628999999999</v>
+        <v>7.3</v>
       </c>
       <c r="B58">
-        <v>7.1078635022837107</v>
-      </c>
-      <c r="C58">
-        <v>-0.49914188792928083</v>
+        <v>0.48268586728628116</v>
       </c>
       <c r="D58">
-        <v>5.9</v>
+        <v>26.653932666666702</v>
       </c>
       <c r="E58">
-        <v>9.8173049624871916E-2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
+        <v>7.8951647838100074</v>
+      </c>
+      <c r="F58">
+        <v>-0.97057093335367473</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A59">
-        <v>29.124999333333299</v>
+        <v>7.4</v>
       </c>
       <c r="B59">
-        <v>8.715948436304144</v>
-      </c>
-      <c r="C59">
-        <v>-1.030586676898219</v>
+        <v>0.48288786576195997</v>
       </c>
       <c r="D59">
-        <v>6</v>
+        <v>29.122796000000001</v>
       </c>
       <c r="E59">
-        <v>0.10200230493448693</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
+        <v>9.56299693449294</v>
+      </c>
+      <c r="F59">
+        <v>-1.3114490143157429</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A60">
-        <v>31.833368</v>
+        <v>7.5</v>
       </c>
       <c r="B60">
-        <v>10.693373629142032</v>
-      </c>
-      <c r="C60">
-        <v>-0.72593082245534601</v>
+        <v>0.48360583706232335</v>
       </c>
       <c r="D60">
-        <v>6.1</v>
+        <v>31.829903999999999</v>
       </c>
       <c r="E60">
-        <v>0.10601181122885438</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
+        <v>11.560536787215897</v>
+      </c>
+      <c r="F60">
+        <v>-0.83897812569828123</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A61">
-        <v>34.786841666666703</v>
+        <v>7.6</v>
       </c>
       <c r="B61">
-        <v>13.034340168314115</v>
-      </c>
-      <c r="C61">
-        <v>-5.4921240774329645E-2</v>
+        <v>0.4848313184791273</v>
       </c>
       <c r="D61">
-        <v>6.2</v>
+        <v>34.782505999999998</v>
       </c>
       <c r="E61">
-        <v>0.11020339983768933</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
+        <v>13.888525386072828</v>
+      </c>
+      <c r="F61">
+        <v>8.4342602707973502E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A62">
-        <v>38.015993333333299</v>
+        <v>7.7</v>
       </c>
       <c r="B62">
-        <v>15.66034266978026</v>
-      </c>
-      <c r="C62">
-        <v>0.25048773009503678</v>
+        <v>0.48655663678618505</v>
       </c>
       <c r="D62">
-        <v>6.3</v>
+        <v>38.0121446666667</v>
       </c>
       <c r="E62">
-        <v>0.11457903969483449</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
+        <v>16.483061784220961</v>
+      </c>
+      <c r="F62">
+        <v>0.66334930678771897</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A63">
-        <v>41.541401333333297</v>
+        <v>7.8</v>
       </c>
       <c r="B63">
-        <v>18.721182229365958</v>
-      </c>
-      <c r="C63">
-        <v>1.228997168086273</v>
+        <v>0.48877484991246872</v>
       </c>
       <c r="D63">
-        <v>6.4</v>
+        <v>41.536471666666699</v>
       </c>
       <c r="E63">
-        <v>0.11914082637305579</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
+        <v>19.484969030141016</v>
+      </c>
+      <c r="F63">
+        <v>1.5192833532998287</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A64">
-        <v>45.414369000000001</v>
+        <v>7.9</v>
       </c>
       <c r="B64">
-        <v>21.708565137281063</v>
-      </c>
-      <c r="C64">
-        <v>0.15103495178143203</v>
+        <v>0.49147969318981133</v>
       </c>
       <c r="D64">
-        <v>6.5</v>
+        <v>45.408605333333298</v>
       </c>
       <c r="E64">
-        <v>0.12389097214811938</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
+        <v>22.487352208054688</v>
+      </c>
+      <c r="F64">
+        <v>0.27009327508249981</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65">
-        <v>49.616305666666698</v>
+        <v>8</v>
       </c>
       <c r="B65">
-        <v>24.892370037112372</v>
-      </c>
-      <c r="C65">
-        <v>-1.0669913781255187</v>
+        <v>0.49466552972325628</v>
       </c>
       <c r="D65">
-        <v>6.6</v>
+        <v>49.610309666666701</v>
       </c>
       <c r="E65">
-        <v>0.12883179696600369</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
+        <v>25.747283557722294</v>
+      </c>
+      <c r="F65">
+        <v>-0.68698020397322412</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66">
-        <v>54.228700666666697</v>
+        <v>8.1</v>
       </c>
       <c r="B66">
-        <v>29.328838533045083</v>
-      </c>
-      <c r="C66">
-        <v>1.0425996615373263</v>
+        <v>0.49832730448117657</v>
       </c>
       <c r="D66">
-        <v>6.7</v>
+        <v>54.223319666666697</v>
       </c>
       <c r="E66">
-        <v>0.13396572020322392</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
+        <v>30.045855604873029</v>
+      </c>
+      <c r="F66">
+        <v>0.88958840024413977</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67">
-        <v>59.256877666666703</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="B67">
-        <v>33.879527476774875</v>
-      </c>
-      <c r="C67">
-        <v>1.7681032442987576</v>
+        <v>0.50246050174537304</v>
       </c>
       <c r="D67">
-        <v>6.8</v>
+        <v>59.250904333333303</v>
       </c>
       <c r="E67">
-        <v>0.13929525312411034</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
+        <v>34.57948834087194</v>
+      </c>
+      <c r="F67">
+        <v>1.5136177364649035</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A68">
-        <v>64.763100666666702</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="B68">
-        <v>37.878981788347424</v>
-      </c>
-      <c r="C68">
-        <v>-0.17011720768539043</v>
+        <v>0.50706110559929263</v>
       </c>
       <c r="D68">
-        <v>6.9</v>
+        <v>64.756259999999997</v>
       </c>
       <c r="E68">
-        <v>0.14482299195082557</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
+        <v>38.728742127681087</v>
+      </c>
+      <c r="F68">
+        <v>-0.13071067496267338</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A69">
-        <v>70.7758556666667</v>
+        <v>8.4</v>
       </c>
       <c r="B69">
-        <v>42.01324913962543</v>
-      </c>
-      <c r="C69">
-        <v>-2.0898660372104731</v>
+        <v>0.51212556316594771</v>
       </c>
       <c r="D69">
-        <v>7</v>
+        <v>70.769128333333299</v>
       </c>
       <c r="E69">
-        <v>0.1505516114722138</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
+        <v>43.113266636568355</v>
+      </c>
+      <c r="F69">
+        <v>-1.7189948266216866</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A70">
-        <v>77.329959666666696</v>
+        <v>8.5</v>
       </c>
       <c r="B70">
-        <v>47.300912636035008</v>
-      </c>
-      <c r="C70">
-        <v>-1.651405636713529</v>
+        <v>0.51765075033666752</v>
       </c>
       <c r="D70">
-        <v>7.1</v>
+        <v>77.322332666666696</v>
       </c>
       <c r="E70">
-        <v>0.15648385912649951</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
+        <v>48.563691951526565</v>
+      </c>
+      <c r="F70">
+        <v>-1.3719959817977039</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A71">
-        <v>84.494202666666695</v>
+        <v>8.6</v>
       </c>
       <c r="B71">
-        <v>53.7772349822202</v>
-      </c>
-      <c r="C71">
-        <v>0.67687975435274672</v>
+        <v>0.52363393975795935</v>
       </c>
       <c r="D71">
-        <v>7.2</v>
+        <v>84.486834000000002</v>
       </c>
       <c r="E71">
-        <v>0.16262254950057894</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
+        <v>55.064150088361053</v>
+      </c>
+      <c r="F71">
+        <v>0.44744367307332727</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A72">
-        <v>92.326205999999999</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="B72">
-        <v>60.355801807649563</v>
-      </c>
-      <c r="C72">
-        <v>2.6854422455522635</v>
+        <v>0.53007277086694915</v>
       </c>
       <c r="D72">
-        <v>7.3</v>
+        <v>92.318579</v>
       </c>
       <c r="E72">
-        <v>0.16897055919536638</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
+        <v>61.784396945187247</v>
+      </c>
+      <c r="F72">
+        <v>2.1032965632713179</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A73">
-        <v>100.90077333333301</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="B73">
-        <v>63.667345295354714</v>
-      </c>
-      <c r="C73">
-        <v>-0.69200310004709498</v>
+        <v>0.53696522178646122</v>
       </c>
       <c r="D73">
-        <v>7.4</v>
+        <v>100.89543</v>
       </c>
       <c r="E73">
-        <v>0.1755308220124962</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
+        <v>65.866319208316099</v>
+      </c>
+      <c r="F73">
+        <v>-0.5753210518466858</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A74">
-        <v>111.000966666667</v>
+        <v>8.9</v>
       </c>
       <c r="B74">
-        <v>69.971886269899429</v>
-      </c>
-      <c r="C74">
-        <v>0.32305514775130317</v>
+        <v>0.54430958290911735</v>
       </c>
       <c r="D74">
-        <v>7.5</v>
+        <v>110.98699000000001</v>
       </c>
       <c r="E74">
-        <v>0.18230632442277614</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
+        <v>72.62716449400007</v>
+      </c>
+      <c r="F74">
+        <v>0.35032216046625592</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A75">
-        <v>117.01837999999999</v>
+        <v>9</v>
       </c>
       <c r="B75">
-        <v>72.83565288287511</v>
-      </c>
-      <c r="C75">
-        <v>2.334654007953427E-2</v>
+        <v>0.55210443201617021</v>
       </c>
       <c r="D75">
-        <v>7.6</v>
+        <v>117.01297</v>
       </c>
       <c r="E75">
-        <v>0.18930010128123206</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
+        <v>75.703083108500067</v>
+      </c>
+      <c r="F75">
+        <v>-5.6710694837080078E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A76">
-        <v>123.378023333333</v>
+        <v>9.1</v>
       </c>
       <c r="B76">
-        <v>75.170711278518596</v>
-      </c>
-      <c r="C76">
-        <v>-0.92248677421563718</v>
+        <v>0.56034861079133946</v>
       </c>
       <c r="D76">
-        <v>7.7</v>
+        <v>123.370866666667</v>
       </c>
       <c r="E76">
-        <v>0.19651523175747562</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
+        <v>78.561498389247618</v>
+      </c>
+      <c r="F76">
+        <v>-0.6823113269396831</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A77">
-        <v>130.071153333333</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="B77">
-        <v>78.668286813677412</v>
-      </c>
-      <c r="C77">
-        <v>-0.29234777323034905</v>
+        <v>0.56904120260295954</v>
       </c>
       <c r="D77">
-        <v>7.8</v>
+        <v>130.063353333333</v>
       </c>
       <c r="E77">
-        <v>0.20395483545353443</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
+        <v>82.301841306003496</v>
+      </c>
+      <c r="F77">
+        <v>-0.15967428255631683</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A78">
-        <v>137.11121</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="B78">
-        <v>82.220287259745874</v>
-      </c>
-      <c r="C78">
-        <v>0.37278365316402107</v>
+        <v>0.578181511439393</v>
       </c>
       <c r="D78">
-        <v>7.9</v>
+        <v>137.10333666666699</v>
       </c>
       <c r="E78">
-        <v>0.21162206868427635</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
+        <v>86.073279768786534</v>
+      </c>
+      <c r="F78">
+        <v>0.38312450321966823</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A79">
-        <v>144.55971</v>
+        <v>9.4</v>
       </c>
       <c r="B79">
-        <v>85.084312201769222</v>
-      </c>
-      <c r="C79">
-        <v>0.15722380062316599</v>
+        <v>0.5877690418931153</v>
       </c>
       <c r="D79">
-        <v>8</v>
+        <v>144.550726666667</v>
       </c>
       <c r="E79">
-        <v>0.21952012089818754</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
+        <v>89.216600775645247</v>
+      </c>
+      <c r="F79">
+        <v>0.17781700518477397</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A80">
-        <v>152.416963333333</v>
+        <v>9.5</v>
       </c>
       <c r="B80">
-        <v>87.871900475758196</v>
-      </c>
-      <c r="C80">
-        <v>-0.15978680112430102</v>
+        <v>0.59780348009826068</v>
       </c>
       <c r="D80">
-        <v>8.1</v>
+        <v>152.40853999999999</v>
       </c>
       <c r="E80">
-        <v>0.22765221121858378</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.45">
+        <v>92.308524824017212</v>
+      </c>
+      <c r="F80">
+        <v>-6.5685687412884317E-2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A81">
-        <v>160.681823333333</v>
+        <v>9.6</v>
       </c>
       <c r="B81">
-        <v>90.754780366084546</v>
-      </c>
-      <c r="C81">
-        <v>-0.38582871710259842</v>
+        <v>0.60828467553484078</v>
       </c>
       <c r="D81">
-        <v>8.1999999999999993</v>
+        <v>160.67290333333301</v>
       </c>
       <c r="E81">
-        <v>0.23602158508737242</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.45">
+        <v>95.417191364868714</v>
+      </c>
+      <c r="F81">
+        <v>-0.26477451652064526</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A82">
-        <v>169.39784</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="B82">
-        <v>94.308071263517007</v>
-      </c>
-      <c r="C82">
-        <v>5.8755972030860838E-2</v>
+        <v>0.61921262362044482</v>
       </c>
       <c r="D82">
-        <v>8.3000000000000007</v>
+        <v>169.38767999999999</v>
       </c>
       <c r="E82">
-        <v>0.24463151099528896</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.45">
+        <v>98.866037061708241</v>
+      </c>
+      <c r="F82">
+        <v>-0.10753631799946127</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A83">
-        <v>178.595476666667</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="B83">
-        <v>97.694030170423289</v>
-      </c>
-      <c r="C83">
-        <v>0.23679976515787787</v>
+        <v>0.63058744901705799</v>
       </c>
       <c r="D83">
-        <v>8.4</v>
+        <v>178.58491333333299</v>
       </c>
       <c r="E83">
-        <v>0.25348527728412668</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.45">
+        <v>102.39460814664976</v>
+      </c>
+      <c r="F83">
+        <v>0.11519206840028327</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A84">
-        <v>188.28131666666701</v>
+        <v>9.9</v>
       </c>
       <c r="B84">
-        <v>100.88319813216532</v>
-      </c>
-      <c r="C84">
-        <v>0.14532005710518506</v>
+        <v>0.64240938958680949</v>
       </c>
       <c r="D84">
-        <v>8.5</v>
+        <v>188.26902000000001</v>
       </c>
       <c r="E84">
-        <v>0.26258618900789271</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.45">
+        <v>105.64453149345267</v>
+      </c>
+      <c r="F84">
+        <v>6.8300251944985194E-2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A85">
-        <v>198.483016666667</v>
+        <v>10</v>
       </c>
       <c r="B85">
-        <v>104.09671470954888</v>
-      </c>
-      <c r="C85">
-        <v>2.0969372603160005E-2</v>
+        <v>0.65467878093603438</v>
       </c>
       <c r="D85">
-        <v>8.6</v>
+        <v>198.473176666667</v>
       </c>
       <c r="E85">
-        <v>0.27193756484107429</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.45">
+        <v>108.76012917044645</v>
+      </c>
+      <c r="F85">
+        <v>-8.7922598098721896E-2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A86">
-        <v>209.25458333333299</v>
+        <v>10.1</v>
       </c>
       <c r="B86">
-        <v>107.49441868086994</v>
-      </c>
-      <c r="C86">
-        <v>1.1604779871246664E-2</v>
+        <v>0.66739604149206733</v>
       </c>
       <c r="D86">
-        <v>8.6999999999999993</v>
+        <v>209.24372666666699</v>
       </c>
       <c r="E86">
-        <v>0.28154273402331564</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.45">
+        <v>112.10879411927012</v>
+      </c>
+      <c r="F86">
+        <v>-1.3636591717974333E-2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A87">
-        <v>220.60282333333299</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="B87">
-        <v>111.1230472844279</v>
-      </c>
-      <c r="C87">
-        <v>0.16309898032976544</v>
+        <v>0.68056165806175595</v>
       </c>
       <c r="D87">
-        <v>8.8000000000000007</v>
+        <v>220.593543333333</v>
       </c>
       <c r="E87">
-        <v>0.29140503333079637</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.45">
+        <v>115.47265207004826</v>
+      </c>
+      <c r="F87">
+        <v>9.6578626979914567E-2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A88">
-        <v>232.565656666667</v>
+        <v>10.3</v>
       </c>
       <c r="B88">
-        <v>114.64610368161505</v>
-      </c>
-      <c r="C88">
-        <v>0.17581340031992387</v>
+        <v>0.69417617182481284</v>
       </c>
       <c r="D88">
-        <v>8.9</v>
+        <v>232.55527333333299</v>
       </c>
       <c r="E88">
-        <v>0.30152780406548085</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.45">
+        <v>118.42824465784814</v>
+      </c>
+      <c r="F88">
+        <v>-0.10761245028462998</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A89">
-        <v>245.18743333333299</v>
+        <v>10.4</v>
       </c>
       <c r="B89">
-        <v>117.65710915146731</v>
-      </c>
-      <c r="C89">
-        <v>-0.27148826934381026</v>
+        <v>0.70824016471888074</v>
       </c>
       <c r="D89">
-        <v>9</v>
+        <v>245.18323333333299</v>
       </c>
       <c r="E89">
-        <v>0.3119143890542026</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.45">
+        <v>121.53913364175342</v>
+      </c>
+      <c r="F89">
+        <v>-0.13235225497130457</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A90">
-        <v>258.49435999999997</v>
+        <v>10.5</v>
       </c>
       <c r="B90">
-        <v>121.04265958731648</v>
-      </c>
-      <c r="C90">
-        <v>-0.39145245427576647</v>
+        <v>0.72275424617659423</v>
       </c>
       <c r="D90">
-        <v>9.1</v>
+        <v>258.47935000000001</v>
       </c>
       <c r="E90">
-        <v>0.3225681296502389</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.45">
+        <v>124.79689709761622</v>
+      </c>
+      <c r="F90">
+        <v>1.9212022434648198E-2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A91">
-        <v>272.49331999999998</v>
+        <v>10.6</v>
       </c>
       <c r="B91">
-        <v>125.04349779882328</v>
-      </c>
-      <c r="C91">
-        <v>2.7116608960577947E-3</v>
+        <v>0.73771904017801471</v>
       </c>
       <c r="D91">
-        <v>9.1999999999999993</v>
+        <v>272.47730000000001</v>
       </c>
       <c r="E91">
-        <v>0.33349236273067162</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.45">
+        <v>128.04908838503715</v>
+      </c>
+      <c r="F91">
+        <v>0.22525209949956518</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A92">
-        <v>287.25715666666702</v>
+        <v>10.7</v>
       </c>
       <c r="B92">
-        <v>129.02301471064433</v>
-      </c>
-      <c r="C92">
-        <v>0.38289293011499353</v>
+        <v>0.75313517258464957</v>
       </c>
       <c r="D92">
-        <v>9.3000000000000007</v>
+        <v>287.21875333333298</v>
       </c>
       <c r="E92">
-        <v>0.34469041768338182</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.45">
+        <v>131.38008831525386</v>
+      </c>
+      <c r="F92">
+        <v>0.55512039658525181</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A93">
-        <v>302.85682333333301</v>
+        <v>10.8</v>
       </c>
       <c r="B93">
-        <v>131.81972912860431</v>
-      </c>
-      <c r="C93">
-        <v>-0.1185218105803614</v>
+        <v>0.76900325872382214</v>
       </c>
       <c r="D93">
-        <v>9.4</v>
+        <v>302.82671333333298</v>
       </c>
       <c r="E93">
-        <v>0.35616561337803637</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="D94">
-        <v>9.5</v>
-      </c>
-      <c r="E94">
-        <v>0.36792125511587476</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="D95">
-        <v>9.6</v>
-      </c>
-      <c r="E95">
-        <v>0.37996063155350879</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="D96">
-        <v>9.6999999999999993</v>
-      </c>
-      <c r="E96">
-        <v>0.3922870115963159</v>
-      </c>
-    </row>
-    <row r="97" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D97">
-        <v>9.8000000000000007</v>
-      </c>
-      <c r="E97">
-        <v>0.40490364125733447</v>
-      </c>
-    </row>
-    <row r="98" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D98">
-        <v>9.9</v>
-      </c>
-      <c r="E98">
-        <v>0.4178137404778629</v>
-      </c>
-    </row>
-    <row r="99" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D99">
-        <v>10</v>
-      </c>
-      <c r="E99">
-        <v>0.4310204999062397</v>
-      </c>
-    </row>
-    <row r="100" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D100">
-        <v>10.1</v>
-      </c>
-      <c r="E100">
-        <v>0.44452707763151178</v>
-      </c>
-    </row>
-    <row r="101" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D101">
-        <v>10.199999999999999</v>
-      </c>
-      <c r="E101">
-        <v>0.45833659586892578</v>
-      </c>
-    </row>
-    <row r="102" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D102">
-        <v>10.3</v>
-      </c>
-      <c r="E102">
-        <v>0.4724933427948097</v>
-      </c>
-    </row>
-    <row r="103" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D103">
-        <v>10.4</v>
-      </c>
-      <c r="E103">
-        <v>0.48720370394474255</v>
-      </c>
-    </row>
-    <row r="104" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D104">
-        <v>10.5</v>
-      </c>
-      <c r="E104">
-        <v>0.50222954325985947</v>
-      </c>
-    </row>
-    <row r="105" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D105">
-        <v>10.6</v>
-      </c>
-      <c r="E105">
-        <v>0.51757229323015064</v>
-      </c>
-    </row>
-    <row r="106" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D106">
-        <v>10.7</v>
-      </c>
-      <c r="E106">
-        <v>0.53323331904581228</v>
-      </c>
-    </row>
-    <row r="107" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D107">
-        <v>10.8</v>
-      </c>
-      <c r="E107">
-        <v>0.5492139204083325</v>
-      </c>
-    </row>
-    <row r="108" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D108">
+        <v>132.69656753224851</v>
+      </c>
+      <c r="F93">
+        <v>-0.57012678269893213</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A94">
         <v>10.9</v>
       </c>
-      <c r="E108">
-        <v>0.56551533330437953</v>
-      </c>
-    </row>
-    <row r="109" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D109">
+      <c r="B94">
+        <v>0.7853238911945124</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A95">
         <v>11</v>
       </c>
-      <c r="E109">
-        <v>0.58213873174291297</v>
-      </c>
-    </row>
-    <row r="110" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D110">
+      <c r="B95">
+        <v>0.80209762786792793</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A96">
         <v>11.1</v>
       </c>
-      <c r="E110">
-        <v>0.59908522945599663</v>
-      </c>
-    </row>
-    <row r="111" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D111">
+      <c r="B96">
+        <v>0.81932498005801102</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A97">
         <v>11.2</v>
       </c>
-      <c r="E111">
-        <v>0.61635588156372501</v>
-      </c>
-    </row>
-    <row r="112" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D112">
+      <c r="B97">
+        <v>0.83700640083888478</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A98">
         <v>11.3</v>
       </c>
-      <c r="E112">
-        <v>0.63395168620373343</v>
-      </c>
-    </row>
-    <row r="113" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D113">
+      <c r="B98">
+        <v>0.85514227348787519</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A99">
         <v>11.4</v>
       </c>
-      <c r="E113">
-        <v>0.65187358612570467</v>
-      </c>
-    </row>
-    <row r="114" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D114">
+      <c r="B99">
+        <v>0.87373290003423476</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A100">
         <v>11.5</v>
       </c>
-      <c r="E114">
-        <v>0.67012247025133975</v>
-      </c>
-    </row>
-    <row r="115" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D115">
+      <c r="B100">
+        <v>0.89277848989508735</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A101">
         <v>11.6</v>
       </c>
-      <c r="E115">
-        <v>0.68869917520020463</v>
-      </c>
-    </row>
-    <row r="116" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D116">
+      <c r="B101">
+        <v>0.91227914858135006</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A102">
         <v>11.7</v>
       </c>
-      <c r="E116">
-        <v>0.70760448678188925</v>
-      </c>
-    </row>
-    <row r="117" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D117">
+      <c r="B102">
+        <v>0.93223486645756504</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A103">
         <v>11.8</v>
       </c>
-      <c r="E117">
-        <v>0.72683914145492745</v>
-      </c>
-    </row>
-    <row r="118" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D118">
+      <c r="B103">
+        <v>0.95264550754063004</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A104">
         <v>11.9</v>
       </c>
-      <c r="E118">
-        <v>0.74640382775286618</v>
-      </c>
-    </row>
-    <row r="119" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D119">
+      <c r="B104">
+        <v>0.97351079832338816</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A105">
         <v>12</v>
       </c>
-      <c r="E119">
-        <v>0.76629918767797134</v>
-      </c>
-    </row>
-    <row r="120" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D120">
+      <c r="B105">
+        <v>0.99483031660995824</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A106">
         <v>12.1</v>
       </c>
-      <c r="E120">
-        <v>0.78652581806292354</v>
-      </c>
-    </row>
-    <row r="121" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D121">
+      <c r="B106">
+        <v>1.0166034803504878</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A107">
         <v>12.2</v>
       </c>
-      <c r="E121">
-        <v>0.80708427190097742</v>
-      </c>
-    </row>
-    <row r="122" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D122">
+      <c r="B107">
+        <v>1.0388295364637985</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A108">
         <v>12.3</v>
       </c>
-      <c r="E122">
-        <v>0.8279750596449833</v>
-      </c>
-    </row>
-    <row r="123" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D123">
+      <c r="B108">
+        <v>1.0615075496370925</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A109">
         <v>12.4</v>
       </c>
-      <c r="E123">
-        <v>0.84919865047567933</v>
-      </c>
-    </row>
-    <row r="124" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D124">
+      <c r="B109">
+        <v>1.0846363910925272</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A110">
         <v>12.5</v>
       </c>
-      <c r="E124">
-        <v>0.87075547353969329</v>
-      </c>
-    </row>
-    <row r="125" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D125">
+      <c r="B110">
+        <v>1.1082147273110912</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A111">
         <v>12.6</v>
       </c>
-      <c r="E125">
-        <v>0.8926459191576297</v>
-      </c>
-    </row>
-    <row r="126" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D126">
+      <c r="B111">
+        <v>1.1322410087047372</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A112">
         <v>12.7</v>
       </c>
-      <c r="E126">
-        <v>0.91487034000269696</v>
-      </c>
-    </row>
-    <row r="127" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D127">
+      <c r="B112">
+        <v>1.1567134582282768</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A113">
         <v>12.8</v>
       </c>
-      <c r="E127">
-        <v>0.93742905225022544</v>
-      </c>
-    </row>
-    <row r="128" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D128">
+      <c r="B113">
+        <v>1.181630059922989</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A114">
         <v>12.9</v>
       </c>
-      <c r="E128">
-        <v>0.96032233669854428</v>
-      </c>
-    </row>
-    <row r="129" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D129">
+      <c r="B114">
+        <v>1.2069885473843458</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A115">
         <v>13</v>
       </c>
-      <c r="E129">
-        <v>0.98355043986155821</v>
-      </c>
-    </row>
-    <row r="130" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D130">
+      <c r="B115">
+        <v>1.2327863921466768</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A116">
         <v>13.1</v>
       </c>
-      <c r="E130">
-        <v>1.0071135750334823</v>
-      </c>
-    </row>
-    <row r="131" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D131">
+      <c r="B116">
+        <v>1.2590207919779479</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A117">
         <v>13.2</v>
       </c>
-      <c r="E131">
-        <v>1.0310119233260679</v>
-      </c>
-    </row>
-    <row r="132" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D132">
+      <c r="B117">
+        <v>1.2856886590782026</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A118">
         <v>13.3</v>
       </c>
-      <c r="E132">
-        <v>1.05524563467878</v>
-      </c>
-    </row>
-    <row r="133" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D133">
+      <c r="B118">
+        <v>1.3127866081755328</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A119">
         <v>13.4</v>
       </c>
-      <c r="E133">
-        <v>1.0798148288422786</v>
-      </c>
-    </row>
-    <row r="134" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D134">
+      <c r="B119">
+        <v>1.3403109445137424</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A120">
         <v>13.5</v>
       </c>
-      <c r="E134">
-        <v>1.1047195963355909</v>
-      </c>
-    </row>
-    <row r="135" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D135">
+      <c r="B120">
+        <v>1.3682576517261589</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A121">
         <v>13.6</v>
       </c>
-      <c r="E135">
-        <v>1.1299599993774001</v>
-      </c>
-    </row>
-    <row r="136" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D136">
+      <c r="B121">
+        <v>1.3966223795903014</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A122">
         <v>13.7</v>
       </c>
-      <c r="E136">
-        <v>1.155536072791796</v>
-      </c>
-    </row>
-    <row r="137" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D137">
+      <c r="B122">
+        <v>1.4254004316583608</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A123">
         <v>13.8</v>
       </c>
-      <c r="E137">
-        <v>1.1814478248888869</v>
-      </c>
-    </row>
-    <row r="138" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D138">
+      <c r="B123">
+        <v>1.4545867527586713</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A124">
         <v>13.9</v>
       </c>
-      <c r="E138">
-        <v>1.2076952383206752</v>
-      </c>
-    </row>
-    <row r="139" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D139">
+      <c r="B124">
+        <v>1.4841759163635651</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A125">
         <v>14</v>
       </c>
-      <c r="E139">
-        <v>1.2342782709125186</v>
-      </c>
-    </row>
-    <row r="140" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D140">
+      <c r="B125">
+        <v>1.5141621118192075</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A126">
         <v>14.1</v>
       </c>
-      <c r="E140">
-        <v>1.2611968564706271</v>
-      </c>
-    </row>
-    <row r="141" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D141">
+      <c r="B126">
+        <v>1.5445391314331678</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A127">
         <v>14.2</v>
       </c>
-      <c r="E141">
-        <v>1.2884509055659026</v>
-      </c>
-    </row>
-    <row r="142" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D142">
+      <c r="B127">
+        <v>1.5750208344373489</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A128">
         <v>14.3</v>
       </c>
-      <c r="E142">
-        <v>1.3160403062945443</v>
-      </c>
-    </row>
-    <row r="143" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D143">
+      <c r="B128">
+        <v>1.6055699343059247</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A129">
         <v>14.4</v>
       </c>
-      <c r="E143">
-        <v>1.343964925015751</v>
-      </c>
-    </row>
-    <row r="144" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D144">
+      <c r="B129">
+        <v>1.636507433306259</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A130">
         <v>14.5</v>
       </c>
-      <c r="E144">
-        <v>1.372224607066906</v>
-      </c>
-    </row>
-    <row r="145" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D145">
+      <c r="B130">
+        <v>1.6678325593352026</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A131">
         <v>14.6</v>
       </c>
-      <c r="E145">
-        <v>1.4008191774566277</v>
-      </c>
-    </row>
-    <row r="146" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D146">
+      <c r="B131">
+        <v>1.6995445396258222</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A132">
         <v>14.7</v>
       </c>
-      <c r="E146">
-        <v>1.4297484415359896</v>
-      </c>
-    </row>
-    <row r="147" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D147">
+      <c r="B132">
+        <v>1.7316425994125286</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A133">
         <v>14.8</v>
       </c>
-      <c r="E147">
-        <v>1.4590121856483405</v>
-      </c>
-    </row>
-    <row r="148" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D148">
+      <c r="B133">
+        <v>1.7641259606411164</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A134">
         <v>14.9</v>
       </c>
-      <c r="E148">
-        <v>1.4886101777580296</v>
-      </c>
-    </row>
-    <row r="149" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D149">
+      <c r="B134">
+        <v>1.7969938407230703</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A135">
         <v>15</v>
       </c>
-      <c r="E149">
-        <v>1.5185421680584312</v>
-      </c>
-    </row>
-    <row r="150" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D150">
+      <c r="B135">
+        <v>1.8302454513335573</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A136">
         <v>15.1</v>
       </c>
-      <c r="E150">
-        <v>1.5488078895595638</v>
-      </c>
-    </row>
-    <row r="151" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D151">
+      <c r="B136">
+        <v>1.863879997252496</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A137">
         <v>15.2</v>
       </c>
-      <c r="E151">
-        <v>1.5794070586557494</v>
-      </c>
-    </row>
-    <row r="152" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D152">
+      <c r="B137">
+        <v>1.8978966752479707</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A138">
         <v>15.3</v>
       </c>
-      <c r="E152">
-        <v>1.6103393756735487</v>
-      </c>
-    </row>
-    <row r="153" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D153">
+      <c r="B138">
+        <v>1.9322946730015664</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A139">
         <v>15.4</v>
       </c>
-      <c r="E153">
-        <v>1.6416045254004037</v>
-      </c>
-    </row>
-    <row r="154" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D154">
+      <c r="B139">
+        <v>1.9670731680748483</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A140">
         <v>15.5</v>
       </c>
-      <c r="E154">
-        <v>1.6732021775943049</v>
-      </c>
-    </row>
-    <row r="155" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D155">
+      <c r="B140">
+        <v>2.0022313269164593</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A141">
         <v>15.6</v>
       </c>
-      <c r="E155">
-        <v>1.7051319874747919</v>
-      </c>
-    </row>
-    <row r="156" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D156">
+      <c r="B141">
+        <v>2.0377683039092571</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A142">
         <v>15.7</v>
       </c>
-      <c r="E156">
-        <v>1.737393596195691</v>
-      </c>
-    </row>
-    <row r="157" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D157">
+      <c r="B142">
+        <v>2.0736832404568117</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A143">
         <v>15.8</v>
       </c>
-      <c r="E157">
-        <v>1.7699866312998609</v>
-      </c>
-    </row>
-    <row r="158" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D158">
+      <c r="B143">
+        <v>2.109975264108733</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A144">
         <v>15.9</v>
       </c>
-      <c r="E158">
-        <v>1.8029107071563264</v>
-      </c>
-    </row>
-    <row r="159" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D159">
+      <c r="B144">
+        <v>2.1466434877242313</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A145">
         <v>16</v>
       </c>
-      <c r="E159">
-        <v>1.8361654253801052</v>
-      </c>
-    </row>
-    <row r="160" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D160">
+      <c r="B145">
+        <v>2.1836870086732865</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A146">
         <v>16.100000000000001</v>
       </c>
-      <c r="E160">
-        <v>1.8697503752350684</v>
-      </c>
-    </row>
-    <row r="161" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D161">
+      <c r="B146">
+        <v>2.2211049080748917</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A147">
         <v>16.2</v>
       </c>
-      <c r="E161">
-        <v>1.9036651340201778</v>
-      </c>
-    </row>
-    <row r="162" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D162">
+      <c r="B147">
+        <v>2.2588962500717154</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A148">
         <v>16.3</v>
       </c>
-      <c r="E162">
-        <v>1.9379092674393712</v>
-      </c>
-    </row>
-    <row r="163" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D163">
+      <c r="B148">
+        <v>2.297060081140736</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A149">
         <v>16.399999999999999</v>
       </c>
-      <c r="E163">
-        <v>1.972482329955495</v>
-      </c>
-    </row>
-    <row r="164" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D164">
+      <c r="B149">
+        <v>2.3355954294390933</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A150">
         <v>16.5</v>
       </c>
-      <c r="E164">
-        <v>2.0073838651285381</v>
-      </c>
-    </row>
-    <row r="165" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D165">
+      <c r="B150">
+        <v>2.3745013041847565</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A151">
         <v>16.600000000000001</v>
       </c>
-      <c r="E165">
-        <v>2.0426134059385004</v>
-      </c>
-    </row>
-    <row r="166" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D166">
+      <c r="B151">
+        <v>2.4137766950713493</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A152">
         <v>16.7</v>
       </c>
-      <c r="E166">
-        <v>2.0781704750932586</v>
-      </c>
-    </row>
-    <row r="167" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D167">
+      <c r="B152">
+        <v>2.4534205717165594</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A153">
         <v>16.8</v>
       </c>
-      <c r="E167">
-        <v>2.1140545853216737</v>
-      </c>
-    </row>
-    <row r="168" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D168">
+      <c r="B153">
+        <v>2.493431883143661</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A154">
         <v>16.899999999999999</v>
       </c>
-      <c r="E168">
-        <v>2.1502652396522786</v>
-      </c>
-    </row>
-    <row r="169" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D169">
+      <c r="B154">
+        <v>2.5338095572954633</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A155">
         <v>17</v>
       </c>
-      <c r="E169">
-        <v>2.1868019316778975</v>
-      </c>
-    </row>
-    <row r="170" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D170">
+      <c r="B155">
+        <v>2.5745525005802428</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A156">
         <v>17.100000000000001</v>
       </c>
-      <c r="E170">
-        <v>2.2236641458063828</v>
-      </c>
-    </row>
-    <row r="171" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D171">
+      <c r="B156">
+        <v>2.6156595974490884</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A157">
         <v>17.2</v>
       </c>
-      <c r="E171">
-        <v>2.2608513574979447</v>
-      </c>
-    </row>
-    <row r="172" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D172">
+      <c r="B157">
+        <v>2.6571297100040465</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A158">
         <v>17.3</v>
       </c>
-      <c r="E172">
-        <v>2.2983630334892382</v>
-      </c>
-    </row>
-    <row r="173" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D173">
+      <c r="B158">
+        <v>2.6989616776365741</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A159">
         <v>17.399999999999999</v>
       </c>
-      <c r="E173">
-        <v>2.33619863200453</v>
-      </c>
-    </row>
-    <row r="174" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D174">
+      <c r="B159">
+        <v>2.7411543166957855</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A160">
         <v>17.5</v>
       </c>
-      <c r="E174">
-        <v>2.3743576029542988</v>
-      </c>
-    </row>
-    <row r="175" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D175">
+      <c r="B160">
+        <v>2.7837064201859234</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A161">
         <v>17.600000000000001</v>
       </c>
-      <c r="E175">
-        <v>2.4128393881215162</v>
-      </c>
-    </row>
-    <row r="176" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D176">
+      <c r="B161">
+        <v>2.8266167574924874</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A162">
         <v>17.7</v>
       </c>
-      <c r="E176">
-        <v>2.4516434213358949</v>
-      </c>
-    </row>
-    <row r="177" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D177">
+      <c r="B162">
+        <v>2.869884074136567</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A163">
         <v>17.8</v>
       </c>
-      <c r="E177">
-        <v>2.4907691286364515</v>
-      </c>
-    </row>
-    <row r="178" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D178">
+      <c r="B163">
+        <v>2.9135070915567813</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A164">
         <v>17.899999999999999</v>
       </c>
-      <c r="E178">
-        <v>2.530215928422574</v>
-      </c>
-    </row>
-    <row r="179" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D179">
+      <c r="B164">
+        <v>2.9574845069183517</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A165">
         <v>18</v>
       </c>
-      <c r="E179">
-        <v>2.5699832315939557</v>
-      </c>
-    </row>
-    <row r="180" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D180">
+      <c r="B165">
+        <v>3.001814992948832</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A166">
         <v>18.100000000000001</v>
       </c>
-      <c r="E180">
-        <v>2.610070441679686</v>
-      </c>
-    </row>
-    <row r="181" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D181">
+      <c r="B166">
+        <v>3.0464971977997664</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A167">
         <v>18.2</v>
       </c>
-      <c r="E181">
-        <v>2.6504769549567126</v>
-      </c>
-    </row>
-    <row r="182" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D182">
+      <c r="B167">
+        <v>3.0915297449340624</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A168">
         <v>18.3</v>
       </c>
-      <c r="E182">
-        <v>2.6912021605579768</v>
-      </c>
-    </row>
-    <row r="183" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D183">
+      <c r="B168">
+        <v>3.1369112330384215</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A169">
         <v>18.399999999999999</v>
       </c>
-      <c r="E183">
-        <v>2.7322454405705825</v>
-      </c>
-    </row>
-    <row r="184" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D184">
+      <c r="B169">
+        <v>3.1826402359601538</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A170">
         <v>18.5</v>
       </c>
-      <c r="E184">
-        <v>2.7736061701240744</v>
-      </c>
-    </row>
-    <row r="185" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D185">
+      <c r="B170">
+        <v>3.2287153026683337</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A171">
         <v>18.600000000000001</v>
       </c>
-      <c r="E185">
-        <v>2.8152837174693581</v>
-      </c>
-    </row>
-    <row r="186" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D186">
+      <c r="B171">
+        <v>3.2751349572382127</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A172">
         <v>18.7</v>
       </c>
-      <c r="E186">
-        <v>2.8572774440482926</v>
-      </c>
-    </row>
-    <row r="187" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D187">
+      <c r="B172">
+        <v>3.3218976988589142</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A173">
         <v>18.8</v>
       </c>
-      <c r="E187">
-        <v>2.8995867045543489</v>
-      </c>
-    </row>
-    <row r="188" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D188">
+      <c r="B173">
+        <v>3.3690020018635911</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A174">
         <v>18.899999999999999</v>
       </c>
-      <c r="E188">
-        <v>2.9422108469845973</v>
-      </c>
-    </row>
-    <row r="189" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D189">
+      <c r="B174">
+        <v>3.4164463157816898</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A175">
         <v>19</v>
       </c>
-      <c r="E189">
-        <v>2.9851492126832162</v>
-      </c>
-    </row>
-    <row r="190" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D190">
+      <c r="B175">
+        <v>3.4642290654128405</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A176">
         <v>19.100000000000001</v>
       </c>
-      <c r="E190">
-        <v>3.0284011363768539</v>
-      </c>
-    </row>
-    <row r="191" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D191">
+      <c r="B176">
+        <v>3.5123486509217754</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A177">
         <v>19.2</v>
       </c>
-      <c r="E191">
-        <v>3.0719659462020474</v>
-      </c>
-    </row>
-    <row r="192" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D192">
+      <c r="B177">
+        <v>3.560803447954028</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A178">
         <v>19.3</v>
       </c>
-      <c r="E192">
-        <v>3.1158429637250094</v>
-      </c>
-    </row>
-    <row r="193" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D193">
+      <c r="B178">
+        <v>3.6095918077716167</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A179">
         <v>19.399999999999999</v>
       </c>
-      <c r="E193">
-        <v>3.160031503953908</v>
-      </c>
-    </row>
-    <row r="194" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D194">
+      <c r="B179">
+        <v>3.658712057408656</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A180">
         <v>19.5</v>
       </c>
-      <c r="E194">
-        <v>3.2045308753441399</v>
-      </c>
-    </row>
-    <row r="195" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D195">
+      <c r="B180">
+        <v>3.7081624998459199</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A181">
         <v>19.600000000000001</v>
       </c>
-      <c r="E195">
-        <v>3.2493403797965086</v>
-      </c>
-    </row>
-    <row r="196" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D196">
+      <c r="B181">
+        <v>3.7579414142044167</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A182">
         <v>19.7</v>
       </c>
-      <c r="E196">
-        <v>3.2944593126488506</v>
-      </c>
-    </row>
-    <row r="197" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D197">
+      <c r="B182">
+        <v>3.8080470559570729</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A183">
         <v>19.8</v>
       </c>
-      <c r="E197">
-        <v>3.3398869626611773</v>
-      </c>
-    </row>
-    <row r="198" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D198">
+      <c r="B183">
+        <v>3.8584776571584527</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A184">
         <v>19.899999999999999</v>
       </c>
-      <c r="E198">
-        <v>3.3856226119946511</v>
-      </c>
-    </row>
-    <row r="199" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D199">
+      <c r="B184">
+        <v>3.9092314266916199</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A185">
         <v>20</v>
       </c>
-      <c r="E199">
-        <v>3.4316655361845769</v>
-      </c>
-    </row>
-    <row r="200" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D200">
+      <c r="B185">
+        <v>3.9603065505322395</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A186">
         <v>25</v>
       </c>
-      <c r="E200">
-        <v>6.1074296073163588</v>
-      </c>
-    </row>
-    <row r="201" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D201">
+      <c r="B186">
+        <v>6.8782188728356681</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A187">
         <v>30</v>
       </c>
-      <c r="E201">
-        <v>9.426975535679313</v>
-      </c>
-    </row>
-    <row r="202" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D202">
+      <c r="B187">
+        <v>10.319604687551148</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A188">
         <v>35</v>
       </c>
-      <c r="E202">
-        <v>13.209244357855166</v>
-      </c>
-    </row>
-    <row r="203" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D203">
+      <c r="B188">
+        <v>14.042720246330489</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A189">
         <v>40</v>
       </c>
-      <c r="E203">
-        <v>17.233864446670012</v>
-      </c>
-    </row>
-    <row r="204" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D204">
+      <c r="B189">
+        <v>17.951066664834006</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A190">
         <v>45</v>
       </c>
-      <c r="E204">
-        <v>21.334119543210335</v>
-      </c>
-    </row>
-    <row r="205" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D205">
+      <c r="B190">
+        <v>22.078508999151602</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A191">
         <v>50</v>
       </c>
-      <c r="E205">
-        <v>25.479391231695558</v>
-      </c>
-    </row>
-    <row r="206" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D206">
+      <c r="B191">
+        <v>26.247271507736397</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A192">
         <v>55</v>
       </c>
-      <c r="E206">
-        <v>29.67852114705315</v>
-      </c>
-    </row>
-    <row r="207" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D207">
+      <c r="B192">
+        <v>30.438416602362732</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A193">
         <v>60</v>
       </c>
-      <c r="E207">
-        <v>33.921698061328009</v>
-      </c>
-    </row>
-    <row r="208" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D208">
+      <c r="B193">
+        <v>34.705688334930841</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A194">
         <v>65</v>
       </c>
-      <c r="E208">
-        <v>38.142041226880238</v>
-      </c>
-    </row>
-    <row r="209" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D209">
+      <c r="B194">
+        <v>38.987558707710583</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A195">
         <v>70</v>
       </c>
-      <c r="E209">
-        <v>42.278879775550728</v>
-      </c>
-    </row>
-    <row r="210" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D210">
+      <c r="B195">
+        <v>43.223309828605778</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A196">
         <v>75</v>
       </c>
-      <c r="E210">
-        <v>46.283922562568094</v>
-      </c>
-    </row>
-    <row r="211" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D211">
+      <c r="B196">
+        <v>47.361566326703084</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A197">
         <v>80</v>
       </c>
-      <c r="E211">
-        <v>50.123214873401757</v>
-      </c>
-    </row>
-    <row r="212" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D212">
+      <c r="B197">
+        <v>51.36392130542356</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A198">
         <v>85</v>
       </c>
-      <c r="E212">
-        <v>53.776443091825541</v>
-      </c>
-    </row>
-    <row r="213" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D213">
+      <c r="B198">
+        <v>55.205218217959889</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A199">
         <v>90</v>
       </c>
-      <c r="E213">
-        <v>57.234901103875714</v>
-      </c>
-    </row>
-    <row r="214" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D214">
+      <c r="B199">
+        <v>58.871984816138507</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A200">
         <v>95</v>
       </c>
-      <c r="E214">
-        <v>60.49899267922919</v>
-      </c>
-    </row>
-    <row r="215" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D215">
+      <c r="B200">
+        <v>62.360096604528884</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A201">
         <v>100</v>
       </c>
-      <c r="E215">
-        <v>63.575771907874795</v>
-      </c>
-    </row>
-    <row r="216" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D216">
+      <c r="B201">
+        <v>65.672330222921801</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A202">
         <v>110</v>
       </c>
-      <c r="E216">
-        <v>69.216203472965049</v>
-      </c>
-    </row>
-    <row r="217" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D217">
+      <c r="B202">
+        <v>71.801912757727877</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A203">
         <v>120</v>
       </c>
-      <c r="E217">
-        <v>74.272609862047204</v>
-      </c>
-    </row>
-    <row r="218" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D218">
+      <c r="B203">
+        <v>77.346862807457356</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A204">
         <v>130</v>
       </c>
-      <c r="E218">
-        <v>78.867631827665306</v>
-      </c>
-    </row>
-    <row r="219" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D219">
+      <c r="B204">
+        <v>82.402802950842769</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A205">
         <v>140</v>
       </c>
-      <c r="E219">
-        <v>83.10953236558376</v>
-      </c>
-    </row>
-    <row r="220" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D220">
+      <c r="B205">
+        <v>87.055306243679269</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A206">
         <v>150</v>
       </c>
-      <c r="E220">
-        <v>87.084360490732394</v>
-      </c>
-    </row>
-    <row r="221" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D221">
+      <c r="B206">
+        <v>91.373130279889963</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A207">
         <v>160</v>
       </c>
-      <c r="E221">
-        <v>90.855403780488714</v>
-      </c>
-    </row>
-    <row r="222" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D222">
+      <c r="B207">
+        <v>95.40813845310096</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A208">
         <v>170</v>
       </c>
-      <c r="E222">
-        <v>94.466155010012201</v>
-      </c>
-    </row>
-    <row r="223" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D223">
+      <c r="B208">
+        <v>99.198029871412018</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A209">
         <v>180</v>
       </c>
-      <c r="E223">
-        <v>97.944500726555134</v>
-      </c>
-    </row>
-    <row r="224" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D224">
+      <c r="B209">
+        <v>102.76976743020531</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A210">
         <v>190</v>
       </c>
-      <c r="E224">
-        <v>101.30689560747182</v>
-      </c>
-    </row>
-    <row r="225" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D225">
+      <c r="B210">
+        <v>106.14272375441476</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A211">
         <v>200</v>
       </c>
-      <c r="E225">
-        <v>104.56195712012835</v>
-      </c>
-    </row>
-    <row r="226" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D226">
+      <c r="B211">
+        <v>109.33119643952196</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A212">
         <v>210</v>
       </c>
-      <c r="E226">
-        <v>107.71330177567617</v>
-      </c>
-    </row>
-    <row r="227" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D227">
+      <c r="B212">
+        <v>112.34625615058356</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A213">
         <v>220</v>
       </c>
-      <c r="E227">
-        <v>110.7616441247082</v>
-      </c>
-    </row>
-    <row r="228" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D228">
+      <c r="B213">
+        <v>115.19702113707216</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A214">
         <v>230</v>
       </c>
-      <c r="E228">
-        <v>113.70626664577931</v>
-      </c>
-    </row>
-    <row r="229" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D229">
+      <c r="B214">
+        <v>117.89148792876283</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A215">
         <v>240</v>
       </c>
-      <c r="E229">
-        <v>116.54599313896964</v>
-      </c>
-    </row>
-    <row r="230" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D230">
+      <c r="B215">
+        <v>120.43704147274306</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A216">
         <v>250</v>
       </c>
-      <c r="E230">
-        <v>119.27979159678328</v>
-      </c>
-    </row>
-    <row r="231" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D231">
+      <c r="B216">
+        <v>122.84074583711345</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A217">
         <v>260</v>
       </c>
-      <c r="E231">
-        <v>121.9071130303852</v>
-      </c>
-    </row>
-    <row r="232" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D232">
+      <c r="B217">
+        <v>125.10949189889699</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A218">
         <v>270</v>
       </c>
-      <c r="E232">
-        <v>124.42805014918348</v>
-      </c>
-    </row>
-    <row r="233" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D233">
+      <c r="B218">
+        <v>127.25005660918555</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A219">
         <v>273.14999999999998</v>
       </c>
-      <c r="E233">
-        <v>125.20021741872074</v>
-      </c>
-    </row>
-    <row r="234" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D234">
+      <c r="B219">
+        <v>127.89885588215739</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A220">
         <v>280</v>
       </c>
-      <c r="E234">
-        <v>126.84337880780868</v>
-      </c>
-    </row>
-    <row r="235" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D235">
+      <c r="B220">
+        <v>129.26911113617541</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A221">
         <v>290</v>
       </c>
-      <c r="E235">
-        <v>129.15452757309129</v>
-      </c>
-    </row>
-    <row r="236" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D236">
+      <c r="B221">
+        <v>131.17320235298948</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A222">
         <v>298.14999999999998</v>
       </c>
-      <c r="E236">
-        <v>130.96243985594947</v>
-      </c>
-    </row>
-    <row r="237" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D237">
+      <c r="B222">
+        <v>132.64445074096011</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A223">
         <v>300</v>
       </c>
-      <c r="E237">
-        <v>131.36350696982285</v>
-      </c>
-    </row>
-    <row r="238" spans="4:5" x14ac:dyDescent="0.45">
-      <c r="D238">
+      <c r="B223">
+        <v>132.96872304199101</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A224">
         <v>305</v>
       </c>
-      <c r="E238">
-        <v>132.43044860821243</v>
+      <c r="B224">
+        <v>133.82771714699084</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added ability to generate tga figures
</commit_message>
<xml_diff>
--- a/test/Figure Data.xlsx
+++ b/test/Figure Data.xlsx
@@ -8,22 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deaco\PycharmProjects\FigureGenerator\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC807817-4839-4CBA-8FE8-6EA1C362E487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE3AB5C9-7920-4489-A51B-B6A58F5F1533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="DyOHCO_3" sheetId="1" r:id="rId1"/>
-    <sheet name="DyOHCO_3⋅0.008H_2O" sheetId="2" r:id="rId2"/>
+    <sheet name="DyOHCO_3⋅0.008H_2O" sheetId="1" r:id="rId1"/>
+    <sheet name="DyOHCO_3" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="A_Cp_Cv">DyOHCO_3⋅0.008H_2O!$T$31</definedName>
-    <definedName name="ad_sub">DyOHCO_3⋅0.008H_2O!$O$2</definedName>
-    <definedName name="Al_sub">DyOHCO_3⋅0.008H_2O!$O$6</definedName>
-    <definedName name="Cu_sub">DyOHCO_3⋅0.008H_2O!$O$4</definedName>
-    <definedName name="Ngr_sub">DyOHCO_3⋅0.008H_2O!$O$8</definedName>
-    <definedName name="Other_sub">DyOHCO_3⋅0.008H_2O!$O$10</definedName>
-    <definedName name="scalingfactor">DyOHCO_3⋅0.008H_2O!$L$6</definedName>
+    <definedName name="A_Cp_Cv">DyOHCO_3!$T$31</definedName>
+    <definedName name="ad_sub">DyOHCO_3!$O$2</definedName>
+    <definedName name="Al_sub">DyOHCO_3!$O$6</definedName>
+    <definedName name="Cu_sub">DyOHCO_3!$O$4</definedName>
+    <definedName name="Ngr_sub">DyOHCO_3!$O$8</definedName>
+    <definedName name="Other_sub">DyOHCO_3!$O$10</definedName>
+    <definedName name="scalingfactor">DyOHCO_3!$L$6</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>